<commit_message>
eaddign revenue and growth
</commit_message>
<xml_diff>
--- a/TWST.xlsx
+++ b/TWST.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\zerrr\Desktop\FinModels\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DA71BA9C-10DF-4F69-88EB-A2766407C6EA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5B77276E-B48E-4A7B-9E95-C42137669669}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" activeTab="1" xr2:uid="{7A10FED2-3E19-44B9-9D40-73F90740EF29}"/>
   </bookViews>
@@ -218,7 +218,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="52" uniqueCount="52">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="55" uniqueCount="55">
   <si>
     <t>Main</t>
   </si>
@@ -378,15 +378,25 @@
   </si>
   <si>
     <t>Q427</t>
+  </si>
+  <si>
+    <t>Revenue Growth</t>
+  </si>
+  <si>
+    <t>Gross Margin</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Tax Rate </t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <numFmts count="2">
+  <numFmts count="3">
     <numFmt numFmtId="164" formatCode="&quot;$&quot;#,##0.0"/>
     <numFmt numFmtId="165" formatCode="0.000;[Red]0.000"/>
+    <numFmt numFmtId="166" formatCode="0.00;[Red]0.00"/>
   </numFmts>
   <fonts count="7" x14ac:knownFonts="1">
     <font>
@@ -488,7 +498,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="13">
+  <cellXfs count="14">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="165" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="165" fontId="0" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyBorder="1"/>
@@ -516,6 +526,7 @@
     <xf numFmtId="9" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="166" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -532,10 +543,6 @@
     </ext>
   </extLst>
 </styleSheet>
-</file>
-
-<file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
-<personList xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main"/>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -978,7 +985,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{53C31551-61C1-4FAC-A3EE-2EABFB95B828}">
-  <dimension ref="A1:AA21"/>
+  <dimension ref="A1:AA40"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="9.140625" style="1"/>
@@ -2120,6 +2127,63 @@
         <v>62.402999999999999</v>
       </c>
     </row>
+    <row r="24" spans="3:22" x14ac:dyDescent="0.25">
+      <c r="C24" s="13" t="s">
+        <v>52</v>
+      </c>
+    </row>
+    <row r="25" spans="3:22" x14ac:dyDescent="0.25">
+      <c r="C25" s="13" t="s">
+        <v>53</v>
+      </c>
+    </row>
+    <row r="26" spans="3:22" x14ac:dyDescent="0.25">
+      <c r="C26" s="13" t="s">
+        <v>54</v>
+      </c>
+    </row>
+    <row r="27" spans="3:22" x14ac:dyDescent="0.25">
+      <c r="C27" s="13"/>
+    </row>
+    <row r="28" spans="3:22" x14ac:dyDescent="0.25">
+      <c r="C28" s="13"/>
+    </row>
+    <row r="29" spans="3:22" x14ac:dyDescent="0.25">
+      <c r="C29" s="13"/>
+    </row>
+    <row r="30" spans="3:22" x14ac:dyDescent="0.25">
+      <c r="C30" s="13"/>
+    </row>
+    <row r="31" spans="3:22" x14ac:dyDescent="0.25">
+      <c r="C31" s="13"/>
+    </row>
+    <row r="32" spans="3:22" x14ac:dyDescent="0.25">
+      <c r="C32" s="13"/>
+    </row>
+    <row r="33" spans="3:3" x14ac:dyDescent="0.25">
+      <c r="C33" s="13"/>
+    </row>
+    <row r="34" spans="3:3" x14ac:dyDescent="0.25">
+      <c r="C34" s="13"/>
+    </row>
+    <row r="35" spans="3:3" x14ac:dyDescent="0.25">
+      <c r="C35" s="13"/>
+    </row>
+    <row r="36" spans="3:3" x14ac:dyDescent="0.25">
+      <c r="C36" s="13"/>
+    </row>
+    <row r="37" spans="3:3" x14ac:dyDescent="0.25">
+      <c r="C37" s="13"/>
+    </row>
+    <row r="38" spans="3:3" x14ac:dyDescent="0.25">
+      <c r="C38" s="13"/>
+    </row>
+    <row r="39" spans="3:3" x14ac:dyDescent="0.25">
+      <c r="C39" s="13"/>
+    </row>
+    <row r="40" spans="3:3" x14ac:dyDescent="0.25">
+      <c r="C40" s="13"/>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <legacyDrawing r:id="rId1"/>

</xml_diff>

<commit_message>
looking at ways to valuing a company that is running at a loss
</commit_message>
<xml_diff>
--- a/TWST.xlsx
+++ b/TWST.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\zerrr\Desktop\FinModels\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{75CCDFF3-21D6-4C99-94FD-749E9CD40568}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D9C33F68-890B-4879-93A9-6C1AE2804D73}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" activeTab="1" xr2:uid="{7A10FED2-3E19-44B9-9D40-73F90740EF29}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" xr2:uid="{7A10FED2-3E19-44B9-9D40-73F90740EF29}"/>
   </bookViews>
   <sheets>
     <sheet name="Main" sheetId="1" r:id="rId1"/>
@@ -40,6 +40,40 @@
 </file>
 
 <file path=xl/comments1.xml><?xml version="1.0" encoding="utf-8"?>
+<comments xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr">
+  <authors>
+    <author>robin zerr</author>
+  </authors>
+  <commentList>
+    <comment ref="F53" authorId="0" shapeId="0" xr:uid="{11000462-69AE-4278-B4BC-E98F2AABF7F2}">
+      <text>
+        <r>
+          <rPr>
+            <b/>
+            <sz val="9"/>
+            <color indexed="81"/>
+            <rFont val="Tahoma"/>
+            <family val="2"/>
+          </rPr>
+          <t>robin zerr:</t>
+        </r>
+        <r>
+          <rPr>
+            <sz val="9"/>
+            <color indexed="81"/>
+            <rFont val="Tahoma"/>
+            <family val="2"/>
+          </rPr>
+          <t xml:space="preserve">
+Assumption: Enter a peer-group median or justified scenario multiple. Do not derive this from negative P/E.</t>
+        </r>
+      </text>
+    </comment>
+  </commentList>
+</comments>
+</file>
+
+<file path=xl/comments2.xml><?xml version="1.0" encoding="utf-8"?>
 <comments xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr">
   <authors>
     <author>robin zerr</author>
@@ -218,7 +252,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="57" uniqueCount="57">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="121" uniqueCount="119">
   <si>
     <t>Main</t>
   </si>
@@ -393,20 +427,260 @@
   </si>
   <si>
     <t xml:space="preserve">Yearly: </t>
+  </si>
+  <si>
+    <t>Bull Case</t>
+  </si>
+  <si>
+    <t>Base Case</t>
+  </si>
+  <si>
+    <t>Bear Case</t>
+  </si>
+  <si>
+    <t>Narratives and Setup</t>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">Sentiment: </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>How do other investors feel about the stock?</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>Positioning:</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> Who owns the stock and how much?</t>
+    </r>
+  </si>
+  <si>
+    <t>Investor</t>
+  </si>
+  <si>
+    <t>Ownership</t>
+  </si>
+  <si>
+    <t>Artisan Partners</t>
+  </si>
+  <si>
+    <t>6.41M</t>
+  </si>
+  <si>
+    <t>ARK Investment Management</t>
+  </si>
+  <si>
+    <t>6.38M</t>
+  </si>
+  <si>
+    <t>Vanguard</t>
+  </si>
+  <si>
+    <t>5.48M</t>
+  </si>
+  <si>
+    <t>BlackRock</t>
+  </si>
+  <si>
+    <t>4.93M</t>
+  </si>
+  <si>
+    <t>EdgePoint Investment Group</t>
+  </si>
+  <si>
+    <t>4.08M</t>
+  </si>
+  <si>
+    <t>William Blair</t>
+  </si>
+  <si>
+    <t>3.81M</t>
+  </si>
+  <si>
+    <t>State Street</t>
+  </si>
+  <si>
+    <t>3.09M</t>
+  </si>
+  <si>
+    <t>View as a high growth piotential
+postive has strong revenue 
+negative: widening net loss and high customer concentration
+Instiutions holding a decent percent of it.</t>
+  </si>
+  <si>
+    <t>Bogey number: The number
+ the company needs to beat for investors to view the quarterly positively</t>
+  </si>
+  <si>
+    <t>The company becomes profitable</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Revenue grows steadily but still operate at a net loss? </t>
+  </si>
+  <si>
+    <t>Revenue declines - Still operating at net loss</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Profit? It currrent looks like the price has spiked from
+a earnings increase of 3mm from expected. I feel like I can
+see how much 3mm over expected correlates to a stock price change </t>
+  </si>
+  <si>
+    <t>Latest earnings on aug
+third. Price was 91$ per
+share</t>
+  </si>
+  <si>
+    <t>august 11th price: 123</t>
+  </si>
+  <si>
+    <t>net change =</t>
+  </si>
+  <si>
+    <t>Reported-estimate/estimate 
+earnings</t>
+  </si>
+  <si>
+    <t>VALUING A LOSS-MAKING COMPANY</t>
+  </si>
+  <si>
+    <t>Recommended sequence</t>
+  </si>
+  <si>
+    <t>Use EV / Revenue while EPS and operating income are negative</t>
+  </si>
+  <si>
+    <t>Forecast revenue growth and gross-margin expansion</t>
+  </si>
+  <si>
+    <t>Forecast R&amp;D and SG&amp;A to determine the break-even year</t>
+  </si>
+  <si>
+    <t>Check cash runway and potential dilution before break-even</t>
+  </si>
+  <si>
+    <t>Use P/E only on normalized earnings after profitability</t>
+  </si>
+  <si>
+    <t>Current valuation snapshot</t>
+  </si>
+  <si>
+    <t>TTM Revenue ($mm)</t>
+  </si>
+  <si>
+    <t>TTM Gross Margin</t>
+  </si>
+  <si>
+    <t>TTM Operating Margin</t>
+  </si>
+  <si>
+    <t>Enterprise Value ($mm)</t>
+  </si>
+  <si>
+    <t>Current EV / TTM Revenue</t>
+  </si>
+  <si>
+    <t>TTM Revenue Growth</t>
+  </si>
+  <si>
+    <t>Selected Forward EV / Revenue</t>
+  </si>
+  <si>
+    <t>Forward Revenue ($mm)</t>
+  </si>
+  <si>
+    <t>Implied Enterprise Value ($mm)</t>
+  </si>
+  <si>
+    <t>Implied Equity Value ($mm)</t>
+  </si>
+  <si>
+    <t>Implied Price / Share</t>
+  </si>
+  <si>
+    <t>How to choose the multiple</t>
+  </si>
+  <si>
+    <t>Peer quality</t>
+  </si>
+  <si>
+    <t>Use companies with similar growth, gross margins, recurring revenue and end markets</t>
+  </si>
+  <si>
+    <t>Growth adjustment</t>
+  </si>
+  <si>
+    <t>Higher sustainable growth can justify a higher revenue multiple</t>
+  </si>
+  <si>
+    <t>Profitability adjustment</t>
+  </si>
+  <si>
+    <t>Stronger margins and a shorter path to break-even support a higher multiple</t>
+  </si>
+  <si>
+    <t>Risk adjustment</t>
+  </si>
+  <si>
+    <t>Cash burn, dilution, customer concentration and execution risk reduce the multiple</t>
+  </si>
+  <si>
+    <t>Cross-check</t>
+  </si>
+  <si>
+    <t>Validate the result with a DCF once long-term margins and cash flow are forecast</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <numFmts count="5">
+  <numFmts count="10">
     <numFmt numFmtId="164" formatCode="&quot;$&quot;#,##0.0"/>
     <numFmt numFmtId="165" formatCode="0.000;[Red]0.000"/>
     <numFmt numFmtId="166" formatCode="0.00;[Red]0.00"/>
-    <numFmt numFmtId="169" formatCode="0.000%"/>
-    <numFmt numFmtId="170" formatCode="0;[Red]0"/>
+    <numFmt numFmtId="167" formatCode="0.000%"/>
+    <numFmt numFmtId="168" formatCode="0;[Red]0"/>
+    <numFmt numFmtId="173" formatCode="#,##0.0;[Red]\(#,##0.0\);\-"/>
+    <numFmt numFmtId="174" formatCode="0.0%"/>
+    <numFmt numFmtId="175" formatCode="0.0%;[Red]\(0.0%\)"/>
+    <numFmt numFmtId="176" formatCode="0.0\x"/>
+    <numFmt numFmtId="177" formatCode="&quot;$&quot;0.00"/>
   </numFmts>
-  <fonts count="7" x14ac:knownFonts="1">
+  <fonts count="9" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -455,16 +729,49 @@
       <name val="Tahoma"/>
       <family val="2"/>
     </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <color rgb="FFFFFFFF"/>
+      <name val="Aptos Narrow"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FF0070C0"/>
+      <name val="Aptos Narrow"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
   </fonts>
-  <fills count="2">
+  <fills count="5">
     <fill>
       <patternFill patternType="none"/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FF1D2330"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFE2E3E5"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFF2CC"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
   </fills>
-  <borders count="4">
+  <borders count="16">
     <border>
       <left/>
       <right/>
@@ -501,12 +808,152 @@
       </bottom>
       <diagonal/>
     </border>
+    <border>
+      <left style="medium">
+        <color indexed="64"/>
+      </left>
+      <right style="medium">
+        <color indexed="64"/>
+      </right>
+      <top style="medium">
+        <color indexed="64"/>
+      </top>
+      <bottom style="medium">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="medium">
+        <color indexed="64"/>
+      </left>
+      <right style="medium">
+        <color indexed="64"/>
+      </right>
+      <top style="medium">
+        <color indexed="64"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="medium">
+        <color indexed="64"/>
+      </left>
+      <right style="medium">
+        <color indexed="64"/>
+      </right>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="medium">
+        <color indexed="64"/>
+      </left>
+      <right style="medium">
+        <color indexed="64"/>
+      </right>
+      <top/>
+      <bottom style="medium">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="medium">
+        <color indexed="64"/>
+      </left>
+      <right/>
+      <top style="medium">
+        <color indexed="64"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="medium">
+        <color indexed="64"/>
+      </left>
+      <right/>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="medium">
+        <color indexed="64"/>
+      </left>
+      <right/>
+      <top/>
+      <bottom style="medium">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="medium">
+        <color indexed="64"/>
+      </right>
+      <top style="medium">
+        <color indexed="64"/>
+      </top>
+      <bottom style="medium">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top/>
+      <bottom style="thick">
+        <color rgb="FF1D2330"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top/>
+      <bottom style="thin">
+        <color rgb="FF808080"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="medium">
+        <color rgb="FF000000"/>
+      </top>
+      <bottom style="medium">
+        <color rgb="FF000000"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color rgb="FFC9A227"/>
+      </left>
+      <right style="thin">
+        <color rgb="FFC9A227"/>
+      </right>
+      <top style="thin">
+        <color rgb="FFC9A227"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="FFC9A227"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="18">
+  <cellXfs count="51">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="165" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="165" fontId="0" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyBorder="1"/>
@@ -533,12 +980,111 @@
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="166" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
-    <xf numFmtId="169" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="167" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="10" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="10" fontId="0" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyBorder="1"/>
-    <xf numFmtId="170" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1"/>
-    <xf numFmtId="170" fontId="0" fillId="0" borderId="3" xfId="0" applyNumberFormat="1" applyBorder="1"/>
-    <xf numFmtId="170" fontId="2" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="168" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1"/>
+    <xf numFmtId="168" fontId="0" fillId="0" borderId="3" xfId="0" applyNumberFormat="1" applyBorder="1"/>
+    <xf numFmtId="168" fontId="2" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="7" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="10" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="7" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="7" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="11" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="10" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="10" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="2" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="173" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="174" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="175" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="176" fontId="2" fillId="0" borderId="14" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="176" fontId="8" fillId="4" borderId="15" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="177" fontId="2" fillId="0" borderId="14" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -555,6 +1101,10 @@
     </ext>
   </extLst>
 </styleSheet>
+</file>
+
+<file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
+<personList xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main"/>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -874,7 +1424,7 @@
 
 <file path=xl/webextensions/taskpanes.xml><?xml version="1.0" encoding="utf-8"?>
 <wetp:taskpanes xmlns:wetp="http://schemas.microsoft.com/office/webextensions/taskpanes/2010/11">
-  <wetp:taskpane dockstate="right" visibility="0" width="350" row="0">
+  <wetp:taskpane dockstate="right" visibility="0" width="350" row="3">
     <wetp:webextensionref xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
   </wetp:taskpane>
 </wetp:taskpanes>
@@ -895,23 +1445,26 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{CDB5E06E-9B2E-4FA3-A49A-3E3DCF1084C7}">
-  <dimension ref="A1:F14"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{CDB5E06E-9B2E-4FA3-A49A-3E3DCF1084C7}">
+  <dimension ref="A1:H58"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="9.140625" style="4"/>
-    <col min="2" max="2" width="25.7109375" style="4" customWidth="1"/>
-    <col min="3" max="4" width="9.140625" style="4"/>
-    <col min="5" max="6" width="15.42578125" style="4" bestFit="1" customWidth="1"/>
-    <col min="7" max="16384" width="9.140625" style="4"/>
+    <col min="1" max="1" width="34.28515625" style="4" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="79.140625" style="4" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="51.28515625" style="4" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="9.140625" style="4"/>
+    <col min="5" max="5" width="29.28515625" style="4" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="20.28515625" style="4" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="12.7109375" style="4" customWidth="1"/>
+    <col min="8" max="16384" width="9.140625" style="4"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A1" s="4" t="s">
         <v>0</v>
       </c>
     </row>
-    <row r="3" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:7" x14ac:dyDescent="0.25">
       <c r="E3" s="4" t="s">
         <v>1</v>
       </c>
@@ -919,7 +1472,7 @@
         <v>124</v>
       </c>
     </row>
-    <row r="4" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:7" x14ac:dyDescent="0.25">
       <c r="E4" s="4" t="s">
         <v>2</v>
       </c>
@@ -927,7 +1480,7 @@
         <v>62707424</v>
       </c>
     </row>
-    <row r="5" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:7" x14ac:dyDescent="0.25">
       <c r="E5" s="4" t="s">
         <v>3</v>
       </c>
@@ -936,7 +1489,7 @@
         <v>7775720576</v>
       </c>
     </row>
-    <row r="6" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:7" x14ac:dyDescent="0.25">
       <c r="E6" s="4" t="s">
         <v>4</v>
       </c>
@@ -945,7 +1498,7 @@
         <v>166839000</v>
       </c>
     </row>
-    <row r="7" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:7" x14ac:dyDescent="0.25">
       <c r="E7" s="4" t="s">
         <v>5</v>
       </c>
@@ -954,7 +1507,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="8" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:7" x14ac:dyDescent="0.25">
       <c r="E8" s="4" t="s">
         <v>6</v>
       </c>
@@ -963,26 +1516,30 @@
         <v>7608881576</v>
       </c>
     </row>
-    <row r="9" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:7" x14ac:dyDescent="0.25">
       <c r="E9" s="5"/>
     </row>
-    <row r="10" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:7" x14ac:dyDescent="0.25">
       <c r="B10" s="6" t="s">
         <v>7</v>
       </c>
     </row>
-    <row r="11" spans="1:6" s="7" customFormat="1" ht="0.95" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="12" spans="1:6" ht="60" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:7" s="7" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="E11" s="7">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="12" spans="1:7" ht="30" x14ac:dyDescent="0.25">
       <c r="B12" s="8" t="s">
         <v>8</v>
       </c>
     </row>
-    <row r="13" spans="1:6" ht="30" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:7" ht="30" x14ac:dyDescent="0.25">
       <c r="B13" s="9" t="s">
         <v>9</v>
       </c>
     </row>
-    <row r="14" spans="1:6" ht="60" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:7" ht="45" x14ac:dyDescent="0.25">
       <c r="B14" s="8" t="s">
         <v>44</v>
       </c>
@@ -990,8 +1547,417 @@
         <v>0.99</v>
       </c>
     </row>
+    <row r="15" spans="1:7" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="B15" s="6"/>
+    </row>
+    <row r="16" spans="1:7" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="B16" s="35" t="s">
+        <v>60</v>
+      </c>
+      <c r="C16" s="38" t="s">
+        <v>61</v>
+      </c>
+      <c r="E16" s="23" t="s">
+        <v>63</v>
+      </c>
+      <c r="F16" s="23" t="s">
+        <v>2</v>
+      </c>
+      <c r="G16" s="23" t="s">
+        <v>64</v>
+      </c>
+    </row>
+    <row r="17" spans="2:8" x14ac:dyDescent="0.25">
+      <c r="B17" s="36"/>
+      <c r="C17" s="26" t="s">
+        <v>79</v>
+      </c>
+      <c r="E17" s="24" t="s">
+        <v>65</v>
+      </c>
+      <c r="F17" s="8" t="s">
+        <v>66</v>
+      </c>
+      <c r="G17" s="25">
+        <v>0.1048</v>
+      </c>
+    </row>
+    <row r="18" spans="2:8" x14ac:dyDescent="0.25">
+      <c r="B18" s="36"/>
+      <c r="C18" s="27"/>
+      <c r="E18" s="24" t="s">
+        <v>67</v>
+      </c>
+      <c r="F18" s="8" t="s">
+        <v>68</v>
+      </c>
+      <c r="G18" s="25">
+        <v>0.1043</v>
+      </c>
+    </row>
+    <row r="19" spans="2:8" x14ac:dyDescent="0.25">
+      <c r="B19" s="36"/>
+      <c r="C19" s="27"/>
+      <c r="E19" s="24" t="s">
+        <v>69</v>
+      </c>
+      <c r="F19" s="8" t="s">
+        <v>70</v>
+      </c>
+      <c r="G19" s="25">
+        <v>8.9499999999999996E-2</v>
+      </c>
+    </row>
+    <row r="20" spans="2:8" s="19" customFormat="1" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="B20" s="36"/>
+      <c r="C20" s="28"/>
+      <c r="E20" s="24" t="s">
+        <v>71</v>
+      </c>
+      <c r="F20" s="8" t="s">
+        <v>72</v>
+      </c>
+      <c r="G20" s="25">
+        <v>8.0500000000000002E-2</v>
+      </c>
+    </row>
+    <row r="21" spans="2:8" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="B21" s="36"/>
+      <c r="C21" s="33" t="s">
+        <v>62</v>
+      </c>
+      <c r="E21" s="24" t="s">
+        <v>73</v>
+      </c>
+      <c r="F21" s="8" t="s">
+        <v>74</v>
+      </c>
+      <c r="G21" s="25">
+        <v>6.6699999999999995E-2</v>
+      </c>
+    </row>
+    <row r="22" spans="2:8" x14ac:dyDescent="0.25">
+      <c r="B22" s="36"/>
+      <c r="C22" s="21"/>
+      <c r="E22" s="24" t="s">
+        <v>75</v>
+      </c>
+      <c r="F22" s="8" t="s">
+        <v>76</v>
+      </c>
+      <c r="G22" s="25">
+        <v>6.2199999999999998E-2</v>
+      </c>
+    </row>
+    <row r="23" spans="2:8" x14ac:dyDescent="0.25">
+      <c r="B23" s="36"/>
+      <c r="C23" s="20"/>
+      <c r="E23" s="24" t="s">
+        <v>77</v>
+      </c>
+      <c r="F23" s="8" t="s">
+        <v>78</v>
+      </c>
+      <c r="G23" s="25">
+        <v>5.0500000000000003E-2</v>
+      </c>
+    </row>
+    <row r="24" spans="2:8" x14ac:dyDescent="0.25">
+      <c r="B24" s="36"/>
+      <c r="C24" s="20"/>
+    </row>
+    <row r="25" spans="2:8" x14ac:dyDescent="0.25">
+      <c r="B25" s="36"/>
+      <c r="C25" s="20"/>
+    </row>
+    <row r="26" spans="2:8" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="B26" s="37"/>
+      <c r="C26" s="22"/>
+    </row>
+    <row r="27" spans="2:8" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="B27" s="18"/>
+      <c r="C27" s="34"/>
+    </row>
+    <row r="28" spans="2:8" ht="75.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="B28" s="39" t="s">
+        <v>80</v>
+      </c>
+      <c r="C28" s="40" t="s">
+        <v>84</v>
+      </c>
+      <c r="E28" s="8" t="s">
+        <v>85</v>
+      </c>
+      <c r="F28" s="4" t="s">
+        <v>86</v>
+      </c>
+      <c r="G28" s="6" t="s">
+        <v>87</v>
+      </c>
+      <c r="H28" s="41">
+        <f>(123-91)/91</f>
+        <v>0.35164835164835168</v>
+      </c>
+    </row>
+    <row r="29" spans="2:8" ht="60.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="C29" s="29"/>
+      <c r="G29" s="23" t="s">
+        <v>88</v>
+      </c>
+      <c r="H29" s="42">
+        <f>(118.4 - 114.55)/114.55</f>
+        <v>3.3609777389786197E-2</v>
+      </c>
+    </row>
+    <row r="30" spans="2:8" x14ac:dyDescent="0.25">
+      <c r="B30" s="21" t="s">
+        <v>57</v>
+      </c>
+      <c r="C30" s="30" t="s">
+        <v>81</v>
+      </c>
+    </row>
+    <row r="31" spans="2:8" x14ac:dyDescent="0.25">
+      <c r="B31" s="20"/>
+      <c r="C31" s="31"/>
+    </row>
+    <row r="32" spans="2:8" x14ac:dyDescent="0.25">
+      <c r="B32" s="20"/>
+      <c r="C32" s="31"/>
+    </row>
+    <row r="33" spans="1:6" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="B33" s="20"/>
+      <c r="C33" s="32"/>
+    </row>
+    <row r="34" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="B34" s="21" t="s">
+        <v>58</v>
+      </c>
+      <c r="C34" s="31" t="s">
+        <v>82</v>
+      </c>
+    </row>
+    <row r="35" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="B35" s="20"/>
+      <c r="C35" s="31"/>
+    </row>
+    <row r="36" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="B36" s="20"/>
+      <c r="C36" s="31"/>
+    </row>
+    <row r="37" spans="1:6" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="B37" s="22"/>
+      <c r="C37" s="32"/>
+    </row>
+    <row r="38" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="B38" s="21" t="s">
+        <v>59</v>
+      </c>
+      <c r="C38" s="21" t="s">
+        <v>83</v>
+      </c>
+    </row>
+    <row r="39" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="B39" s="20"/>
+      <c r="C39" s="20"/>
+    </row>
+    <row r="40" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="B40" s="20"/>
+      <c r="C40" s="20"/>
+    </row>
+    <row r="41" spans="1:6" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="B41" s="22"/>
+      <c r="C41" s="22"/>
+    </row>
+    <row r="43" spans="1:6" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A43" s="43" t="s">
+        <v>89</v>
+      </c>
+    </row>
+    <row r="44" spans="1:6" ht="15.75" thickTop="1" x14ac:dyDescent="0.25"/>
+    <row r="45" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A45" s="44" t="s">
+        <v>90</v>
+      </c>
+      <c r="E45" s="44" t="s">
+        <v>96</v>
+      </c>
+    </row>
+    <row r="46" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A46" s="4">
+        <v>1</v>
+      </c>
+      <c r="B46" s="4" t="s">
+        <v>91</v>
+      </c>
+      <c r="E46" s="4" t="s">
+        <v>97</v>
+      </c>
+      <c r="F46" s="45">
+        <f>SUM(Model!S6:V6)</f>
+        <v>431.798</v>
+      </c>
+    </row>
+    <row r="47" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A47" s="4">
+        <v>2</v>
+      </c>
+      <c r="B47" s="4" t="s">
+        <v>92</v>
+      </c>
+      <c r="E47" s="4" t="s">
+        <v>98</v>
+      </c>
+      <c r="F47" s="46">
+        <f>SUM(Model!S12:V12)/SUM(Model!S6:V6)</f>
+        <v>0.51965270797919394</v>
+      </c>
+    </row>
+    <row r="48" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A48" s="4">
+        <v>3</v>
+      </c>
+      <c r="B48" s="4" t="s">
+        <v>93</v>
+      </c>
+      <c r="E48" s="4" t="s">
+        <v>99</v>
+      </c>
+      <c r="F48" s="47">
+        <f>SUM(Model!S13:V13)/SUM(Model!S6:V6)</f>
+        <v>-0.31906817539682908</v>
+      </c>
+    </row>
+    <row r="49" spans="1:6" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A49" s="4">
+        <v>4</v>
+      </c>
+      <c r="B49" s="4" t="s">
+        <v>94</v>
+      </c>
+      <c r="E49" s="4" t="s">
+        <v>100</v>
+      </c>
+      <c r="F49" s="45">
+        <f>F8/1000000</f>
+        <v>7608.8815759999998</v>
+      </c>
+    </row>
+    <row r="50" spans="1:6" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A50" s="4">
+        <v>5</v>
+      </c>
+      <c r="B50" s="4" t="s">
+        <v>95</v>
+      </c>
+      <c r="E50" s="4" t="s">
+        <v>101</v>
+      </c>
+      <c r="F50" s="48">
+        <f>F49/F46</f>
+        <v>17.621391428399392</v>
+      </c>
+    </row>
+    <row r="51" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="E51" s="4" t="s">
+        <v>102</v>
+      </c>
+      <c r="F51" s="46">
+        <f>SUM(Model!S6:V6)/SUM(Model!O6:R6)-1</f>
+        <v>0.19191328086829529</v>
+      </c>
+    </row>
+    <row r="53" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A53" s="44" t="s">
+        <v>108</v>
+      </c>
+      <c r="E53" s="4" t="s">
+        <v>103</v>
+      </c>
+      <c r="F53" s="49"/>
+    </row>
+    <row r="54" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A54" s="4" t="s">
+        <v>109</v>
+      </c>
+      <c r="B54" s="4" t="s">
+        <v>110</v>
+      </c>
+      <c r="E54" s="4" t="s">
+        <v>104</v>
+      </c>
+      <c r="F54" s="45">
+        <f>F46*(1+F51)</f>
+        <v>514.66577085236815</v>
+      </c>
+    </row>
+    <row r="55" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A55" s="4" t="s">
+        <v>111</v>
+      </c>
+      <c r="B55" s="4" t="s">
+        <v>112</v>
+      </c>
+      <c r="E55" s="4" t="s">
+        <v>105</v>
+      </c>
+      <c r="F55" s="45" t="str">
+        <f>IF(F53="","",F53*F54)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="56" spans="1:6" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A56" s="4" t="s">
+        <v>113</v>
+      </c>
+      <c r="B56" s="4" t="s">
+        <v>114</v>
+      </c>
+      <c r="E56" s="4" t="s">
+        <v>106</v>
+      </c>
+      <c r="F56" s="45" t="str">
+        <f>IF(F55="","",F55+F6/1000000-F7/1000000)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="57" spans="1:6" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A57" s="4" t="s">
+        <v>115</v>
+      </c>
+      <c r="B57" s="4" t="s">
+        <v>116</v>
+      </c>
+      <c r="E57" s="4" t="s">
+        <v>107</v>
+      </c>
+      <c r="F57" s="50" t="str">
+        <f>IF(F56="","",F56/(F4/1000000))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="58" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A58" s="4" t="s">
+        <v>117</v>
+      </c>
+      <c r="B58" s="4" t="s">
+        <v>118</v>
+      </c>
+    </row>
   </sheetData>
+  <mergeCells count="9">
+    <mergeCell ref="C22:C26"/>
+    <mergeCell ref="B16:B26"/>
+    <mergeCell ref="C38:C41"/>
+    <mergeCell ref="B30:B33"/>
+    <mergeCell ref="B34:B37"/>
+    <mergeCell ref="B38:B41"/>
+    <mergeCell ref="C30:C33"/>
+    <mergeCell ref="C34:C37"/>
+    <mergeCell ref="C17:C20"/>
+  </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <legacyDrawing r:id="rId1"/>
 </worksheet>
 </file>
 
@@ -1885,7 +2851,7 @@
         <v>-34.739999999999995</v>
       </c>
     </row>
-    <row r="17" spans="3:22" x14ac:dyDescent="0.25">
+    <row r="17" spans="3:26" x14ac:dyDescent="0.25">
       <c r="C17" s="1" t="s">
         <v>39</v>
       </c>
@@ -1947,7 +2913,7 @@
         <v>-0.311</v>
       </c>
     </row>
-    <row r="18" spans="3:22" x14ac:dyDescent="0.25">
+    <row r="18" spans="3:26" x14ac:dyDescent="0.25">
       <c r="C18" s="3" t="s">
         <v>41</v>
       </c>
@@ -2028,11 +2994,14 @@
         <v>-35.050999999999995</v>
       </c>
     </row>
-    <row r="19" spans="3:22" x14ac:dyDescent="0.25">
+    <row r="19" spans="3:26" x14ac:dyDescent="0.25">
       <c r="C19" s="3"/>
       <c r="D19" s="1"/>
-    </row>
-    <row r="20" spans="3:22" x14ac:dyDescent="0.25">
+      <c r="Z19" s="1" t="s">
+        <v>55</v>
+      </c>
+    </row>
+    <row r="20" spans="3:26" x14ac:dyDescent="0.25">
       <c r="C20" s="3" t="s">
         <v>42</v>
       </c>
@@ -2113,7 +3082,7 @@
         <v>-0.56168773937150451</v>
       </c>
     </row>
-    <row r="21" spans="3:22" x14ac:dyDescent="0.25">
+    <row r="21" spans="3:26" x14ac:dyDescent="0.25">
       <c r="C21" s="1" t="s">
         <v>43</v>
       </c>
@@ -2175,7 +3144,7 @@
         <v>62.402999999999999</v>
       </c>
     </row>
-    <row r="24" spans="3:22" x14ac:dyDescent="0.25">
+    <row r="24" spans="3:26" x14ac:dyDescent="0.25">
       <c r="C24" s="11" t="s">
         <v>54</v>
       </c>
@@ -2243,12 +3212,12 @@
         <v>0.18854328580117594</v>
       </c>
     </row>
-    <row r="25" spans="3:22" x14ac:dyDescent="0.25">
+    <row r="25" spans="3:26" x14ac:dyDescent="0.25">
       <c r="C25" s="11" t="s">
         <v>52</v>
       </c>
       <c r="D25" s="12">
-        <f t="shared" ref="D25:H25" si="7">D12/D6</f>
+        <f t="shared" ref="D25:G25" si="7">D12/D6</f>
         <v>0.35608548717216432</v>
       </c>
       <c r="E25" s="12">
@@ -2324,7 +3293,7 @@
         <v>0.52759005203757525</v>
       </c>
     </row>
-    <row r="26" spans="3:22" s="13" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="26" spans="3:26" s="13" customFormat="1" x14ac:dyDescent="0.25">
       <c r="C26" s="13" t="s">
         <v>53</v>
       </c>
@@ -2386,22 +3355,22 @@
         <v>0</v>
       </c>
     </row>
-    <row r="27" spans="3:22" x14ac:dyDescent="0.25">
+    <row r="27" spans="3:26" x14ac:dyDescent="0.25">
       <c r="C27" s="11"/>
     </row>
-    <row r="28" spans="3:22" x14ac:dyDescent="0.25">
+    <row r="28" spans="3:26" x14ac:dyDescent="0.25">
       <c r="C28" s="11"/>
     </row>
-    <row r="29" spans="3:22" x14ac:dyDescent="0.25">
+    <row r="29" spans="3:26" x14ac:dyDescent="0.25">
       <c r="C29" s="11"/>
     </row>
-    <row r="30" spans="3:22" x14ac:dyDescent="0.25">
+    <row r="30" spans="3:26" x14ac:dyDescent="0.25">
       <c r="C30" s="11"/>
     </row>
-    <row r="31" spans="3:22" x14ac:dyDescent="0.25">
+    <row r="31" spans="3:26" x14ac:dyDescent="0.25">
       <c r="C31" s="11"/>
     </row>
-    <row r="32" spans="3:22" x14ac:dyDescent="0.25">
+    <row r="32" spans="3:26" x14ac:dyDescent="0.25">
       <c r="C32" s="11"/>
     </row>
     <row r="33" spans="3:3" x14ac:dyDescent="0.25">

</xml_diff>